<commit_message>
sync excel/2026/实时现货_发电侧小时电价.xlsx from private
</commit_message>
<xml_diff>
--- a/excel/2026/实时现货_发电侧小时电价.xlsx
+++ b/excel/2026/实时现货_发电侧小时电价.xlsx
@@ -1194,7 +1194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z286"/>
+  <dimension ref="A1:Z291"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:26">
@@ -23963,6 +23963,391 @@
         <v>474.26</v>
       </c>
     </row>
+    <row r="287" spans="1:26">
+      <c r="A287" s="2">
+        <v>46310</v>
+      </c>
+      <c r="C287">
+        <v>81.5</v>
+      </c>
+      <c r="D287">
+        <v>0</v>
+      </c>
+      <c r="E287">
+        <v>-2.5</v>
+      </c>
+      <c r="F287">
+        <v>0</v>
+      </c>
+      <c r="G287">
+        <v>202.55</v>
+      </c>
+      <c r="H287">
+        <v>400.01</v>
+      </c>
+      <c r="I287">
+        <v>497.97</v>
+      </c>
+      <c r="J287">
+        <v>464.96</v>
+      </c>
+      <c r="K287">
+        <v>228.56</v>
+      </c>
+      <c r="L287">
+        <v>354.67</v>
+      </c>
+      <c r="M287">
+        <v>344.57</v>
+      </c>
+      <c r="N287">
+        <v>299.48</v>
+      </c>
+      <c r="O287">
+        <v>250.8</v>
+      </c>
+      <c r="P287">
+        <v>346.57</v>
+      </c>
+      <c r="Q287">
+        <v>365.65</v>
+      </c>
+      <c r="R287">
+        <v>485.51</v>
+      </c>
+      <c r="S287">
+        <v>655.5700000000001</v>
+      </c>
+      <c r="T287">
+        <v>823.65</v>
+      </c>
+      <c r="U287">
+        <v>856.92</v>
+      </c>
+      <c r="V287">
+        <v>602.49</v>
+      </c>
+      <c r="W287">
+        <v>782.0700000000001</v>
+      </c>
+      <c r="X287">
+        <v>583.76</v>
+      </c>
+      <c r="Y287">
+        <v>494.88</v>
+      </c>
+      <c r="Z287">
+        <v>497.25</v>
+      </c>
+    </row>
+    <row r="288" spans="1:26">
+      <c r="A288" s="2">
+        <v>46311</v>
+      </c>
+      <c r="C288">
+        <v>492.92</v>
+      </c>
+      <c r="D288">
+        <v>492.22</v>
+      </c>
+      <c r="E288">
+        <v>493.5</v>
+      </c>
+      <c r="F288">
+        <v>493.17</v>
+      </c>
+      <c r="G288">
+        <v>493.58</v>
+      </c>
+      <c r="H288">
+        <v>496.66</v>
+      </c>
+      <c r="I288">
+        <v>496.01</v>
+      </c>
+      <c r="J288">
+        <v>480.2</v>
+      </c>
+      <c r="K288">
+        <v>442.56</v>
+      </c>
+      <c r="L288">
+        <v>261.1</v>
+      </c>
+      <c r="M288">
+        <v>42</v>
+      </c>
+      <c r="N288">
+        <v>-20.4</v>
+      </c>
+      <c r="O288">
+        <v>-60</v>
+      </c>
+      <c r="P288">
+        <v>386.92</v>
+      </c>
+      <c r="Q288">
+        <v>416.74</v>
+      </c>
+      <c r="R288">
+        <v>465.57</v>
+      </c>
+      <c r="S288">
+        <v>482.22</v>
+      </c>
+      <c r="T288">
+        <v>475.75</v>
+      </c>
+      <c r="U288">
+        <v>467.76</v>
+      </c>
+      <c r="V288">
+        <v>472.15</v>
+      </c>
+      <c r="W288">
+        <v>471.9</v>
+      </c>
+      <c r="X288">
+        <v>545.41</v>
+      </c>
+      <c r="Y288">
+        <v>530.6</v>
+      </c>
+      <c r="Z288">
+        <v>580.0599999999999</v>
+      </c>
+    </row>
+    <row r="289" spans="1:26">
+      <c r="A289" s="2">
+        <v>46312</v>
+      </c>
+      <c r="C289">
+        <v>709.77</v>
+      </c>
+      <c r="D289">
+        <v>776.01</v>
+      </c>
+      <c r="E289">
+        <v>749.11</v>
+      </c>
+      <c r="F289">
+        <v>728.23</v>
+      </c>
+      <c r="G289">
+        <v>800.11</v>
+      </c>
+      <c r="H289">
+        <v>721.1799999999999</v>
+      </c>
+      <c r="I289">
+        <v>610.96</v>
+      </c>
+      <c r="J289">
+        <v>597.39</v>
+      </c>
+      <c r="K289">
+        <v>791.6900000000001</v>
+      </c>
+      <c r="L289">
+        <v>964.8200000000001</v>
+      </c>
+      <c r="M289">
+        <v>1046.71</v>
+      </c>
+      <c r="N289">
+        <v>1102</v>
+      </c>
+      <c r="O289">
+        <v>1212.42</v>
+      </c>
+      <c r="P289">
+        <v>1067.58</v>
+      </c>
+      <c r="Q289">
+        <v>920.3099999999999</v>
+      </c>
+      <c r="R289">
+        <v>842.1</v>
+      </c>
+      <c r="S289">
+        <v>975.48</v>
+      </c>
+      <c r="T289">
+        <v>871.98</v>
+      </c>
+      <c r="U289">
+        <v>911.79</v>
+      </c>
+      <c r="V289">
+        <v>997.1799999999999</v>
+      </c>
+      <c r="W289">
+        <v>1020.24</v>
+      </c>
+      <c r="X289">
+        <v>936.16</v>
+      </c>
+      <c r="Y289">
+        <v>963.41</v>
+      </c>
+      <c r="Z289">
+        <v>881.12</v>
+      </c>
+    </row>
+    <row r="290" spans="1:26">
+      <c r="A290" s="2">
+        <v>46313</v>
+      </c>
+      <c r="C290">
+        <v>474.9</v>
+      </c>
+      <c r="D290">
+        <v>435.36</v>
+      </c>
+      <c r="E290">
+        <v>405.37</v>
+      </c>
+      <c r="F290">
+        <v>371.23</v>
+      </c>
+      <c r="G290">
+        <v>147.49</v>
+      </c>
+      <c r="H290">
+        <v>22.73</v>
+      </c>
+      <c r="I290">
+        <v>71.33</v>
+      </c>
+      <c r="J290">
+        <v>-20.99</v>
+      </c>
+      <c r="K290">
+        <v>-80</v>
+      </c>
+      <c r="L290">
+        <v>-80</v>
+      </c>
+      <c r="M290">
+        <v>-80</v>
+      </c>
+      <c r="N290">
+        <v>-80</v>
+      </c>
+      <c r="O290">
+        <v>-80</v>
+      </c>
+      <c r="P290">
+        <v>-80</v>
+      </c>
+      <c r="Q290">
+        <v>-80</v>
+      </c>
+      <c r="R290">
+        <v>81.02</v>
+      </c>
+      <c r="S290">
+        <v>549.78</v>
+      </c>
+      <c r="T290">
+        <v>516.34</v>
+      </c>
+      <c r="U290">
+        <v>535.4400000000001</v>
+      </c>
+      <c r="V290">
+        <v>504.75</v>
+      </c>
+      <c r="W290">
+        <v>507.85</v>
+      </c>
+      <c r="X290">
+        <v>509.17</v>
+      </c>
+      <c r="Y290">
+        <v>549.38</v>
+      </c>
+      <c r="Z290">
+        <v>655.42</v>
+      </c>
+    </row>
+    <row r="291" spans="1:26">
+      <c r="A291" s="2">
+        <v>46314</v>
+      </c>
+      <c r="C291">
+        <v>466</v>
+      </c>
+      <c r="D291">
+        <v>462.73</v>
+      </c>
+      <c r="E291">
+        <v>465.69</v>
+      </c>
+      <c r="F291">
+        <v>467.83</v>
+      </c>
+      <c r="G291">
+        <v>467.05</v>
+      </c>
+      <c r="H291">
+        <v>467.55</v>
+      </c>
+      <c r="I291">
+        <v>467.52</v>
+      </c>
+      <c r="J291">
+        <v>460.61</v>
+      </c>
+      <c r="K291">
+        <v>418.84</v>
+      </c>
+      <c r="L291">
+        <v>403.16</v>
+      </c>
+      <c r="M291">
+        <v>446.14</v>
+      </c>
+      <c r="N291">
+        <v>468.33</v>
+      </c>
+      <c r="O291">
+        <v>463.64</v>
+      </c>
+      <c r="P291">
+        <v>512.75</v>
+      </c>
+      <c r="Q291">
+        <v>582.55</v>
+      </c>
+      <c r="R291">
+        <v>502.01</v>
+      </c>
+      <c r="S291">
+        <v>462.34</v>
+      </c>
+      <c r="T291">
+        <v>463.67</v>
+      </c>
+      <c r="U291">
+        <v>460.68</v>
+      </c>
+      <c r="V291">
+        <v>454.92</v>
+      </c>
+      <c r="W291">
+        <v>452.5</v>
+      </c>
+      <c r="X291">
+        <v>447.03</v>
+      </c>
+      <c r="Y291">
+        <v>453.51</v>
+      </c>
+      <c r="Z291">
+        <v>447.34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>